<commit_message>
Remover folha extra do template Excel
</commit_message>
<xml_diff>
--- a/public/ATT_IMPORT.xlsx
+++ b/public/ATT_IMPORT.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\trilhos-model-export\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SellForge-Shipping - Cópia\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CFC4833-6682-4A31-B346-425952DA1958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394D64E6-7DFA-4C03-AAE3-005D55EAF76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11160" yWindow="1920" windowWidth="17085" windowHeight="13035" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha1" sheetId="1" r:id="rId1"/>
-    <sheet name="Folha4" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Folha1!$A$1:$O$1</definedName>
@@ -83,7 +82,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,12 +95,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF222222"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -124,12 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -485,7 +475,7 @@
   <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.85546875" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="2" customWidth="1"/>
     <col min="3" max="3" width="30.28515625" customWidth="1"/>
     <col min="4" max="4" width="32.28515625" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" customWidth="1"/>
@@ -503,7 +493,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -577,108 +567,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB69A9D6-FD31-4060-B317-D6D98743426D}">
-  <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-    </row>
-    <row r="9" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-    </row>
-    <row r="17" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
-    </row>
-    <row r="29" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B30" s="2"/>
-    </row>
-    <row r="31" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B31" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>